<commit_message>
[Feat] 콘텐츠 데이터 ScriptObject 연결
</commit_message>
<xml_diff>
--- a/Assets/Excel/ItemExcel.xlsx
+++ b/Assets/Excel/ItemExcel.xlsx
@@ -5,7 +5,7 @@
   <workbookPr codeName="현재_통합_문서" defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\103-28\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Git\2026_01_2_B_GameProject\Assets\Excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="8_{D6539941-DA6A-453D-BA05-E7A973DE362C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
@@ -734,19 +734,11 @@
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="문서" ma:contentTypeID="0x01010085E50190E5AC1447B19EDBA1B05CF469" ma:contentTypeVersion="5" ma:contentTypeDescription="새 문서를 만듭니다." ma:contentTypeScope="" ma:versionID="9192ac93929c2a48cb37d04dd173a6fe">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns3="00044592-a025-42cc-9a6e-0f23f3673bb9" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="93df2b162b379f41546994998a9e54ab" ns3:_="">
     <xsd:import namespace="00044592-a025-42cc-9a6e-0f23f3673bb9"/>
@@ -896,6 +888,15 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
@@ -905,14 +906,6 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A0A3616E-E682-4DCD-9381-B65A4F51BE67}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1A0B6191-CAC8-4C6D-95E1-A1E3BB63D290}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -930,6 +923,14 @@
 </ds:datastoreItem>
 </file>
 
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A0A3616E-E682-4DCD-9381-B65A4F51BE67}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8AC39420-0373-4A09-9946-2D1CD8099C63}">
   <ds:schemaRefs>

</xml_diff>